<commit_message>
Add File2 trial capping Ø1200 at Q_plein (~4.93 m3/s)
Compose/Calcul_QpleinCap use MIN(FHWA, Q_plein) so routing cannot
exceed Manning full-pipe capacity; Parametres column D shows WSEmax.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Retention_1200_File4_TimeSeries.xlsx
+++ b/engineering/drainage-design/retention_volume/Retention_1200_File4_TimeSeries.xlsx
@@ -3526,7 +3526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3539,7 +3539,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Colonnes = formules Excel. Crest / facteur pipe en jaune.</t>
+          <t>Colonnes = formules Excel. Crest / facteur pipe / plafond Q en jaune.</t>
         </is>
       </c>
     </row>
@@ -3633,142 +3633,72 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Q_cap (m3/s)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>1E9</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>WSE</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>HW</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>y_ov</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>A_ditch</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>V_ditch</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>V_pond</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>V_total</t>
         </is>
       </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>Q_1200</t>
         </is>
       </c>
-      <c r="I12" s="14" t="inlineStr">
+      <c r="I14" s="14" t="inlineStr">
         <is>
           <t>Q_overflow</t>
         </is>
       </c>
-      <c r="J12" s="14" t="inlineStr">
+      <c r="J14" s="14" t="inlineStr">
         <is>
           <t>Qout</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="n">
-        <v>34.88</v>
-      </c>
-      <c r="B13" s="18">
-        <f>A13-$B$10</f>
-        <v/>
-      </c>
-      <c r="C13" s="18">
-        <f>MAX(0,A13-$B$4)</f>
-        <v/>
-      </c>
-      <c r="D13" s="16">
-        <f>IF(C13&lt;=0,0,($B$5+$B$7*C13)*C13)</f>
-        <v/>
-      </c>
-      <c r="E13" s="15">
-        <f>D13*$B$9</f>
-        <v/>
-      </c>
-      <c r="F13" s="15">
-        <f>IF(A13&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A13&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A13,Stage_Storage!$A$11:$A$18,1))+(A13-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A13,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A13,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A13,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A13,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A13,Stage_Storage!$A$11:$A$18,1)))))</f>
-        <v/>
-      </c>
-      <c r="G13" s="12">
-        <f>E13+F13</f>
-        <v/>
-      </c>
-      <c r="H13" s="16">
-        <f>($B$11)*(IF(B13&lt;=0,0,IF(B13&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B13,Courbe_QH_1200!$A$20:$A$80,1))+(B13-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B13,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B13,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B13,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B13,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B13,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
-        <v/>
-      </c>
-      <c r="I13" s="16">
-        <f>IF(C13&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D13*IF(($B$5+2*C13*SQRT(1+$B$7^2))&lt;=0,0,((D13/($B$5+2*C13*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
-        <v/>
-      </c>
-      <c r="J13" s="8">
-        <f>H13+I13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="n">
-        <v>34.98</v>
-      </c>
-      <c r="B14" s="18">
-        <f>A14-$B$10</f>
-        <v/>
-      </c>
-      <c r="C14" s="18">
-        <f>MAX(0,A14-$B$4)</f>
-        <v/>
-      </c>
-      <c r="D14" s="16">
-        <f>IF(C14&lt;=0,0,($B$5+$B$7*C14)*C14)</f>
-        <v/>
-      </c>
-      <c r="E14" s="15">
-        <f>D14*$B$9</f>
-        <v/>
-      </c>
-      <c r="F14" s="15">
-        <f>IF(A14&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A14&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A14,Stage_Storage!$A$11:$A$18,1))+(A14-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A14,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A14,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A14,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A14,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A14,Stage_Storage!$A$11:$A$18,1)))))</f>
-        <v/>
-      </c>
-      <c r="G14" s="12">
-        <f>E14+F14</f>
-        <v/>
-      </c>
-      <c r="H14" s="16">
-        <f>($B$11)*(IF(B14&lt;=0,0,IF(B14&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B14,Courbe_QH_1200!$A$20:$A$80,1))+(B14-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B14,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B14,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B14,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B14,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B14,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
-        <v/>
-      </c>
-      <c r="I14" s="16">
-        <f>IF(C14&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D14*IF(($B$5+2*C14*SQRT(1+$B$7^2))&lt;=0,0,((D14/($B$5+2*C14*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
-        <v/>
-      </c>
-      <c r="J14" s="8">
-        <f>H14+I14</f>
-        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="n">
-        <v>35.08</v>
+        <v>34.88</v>
       </c>
       <c r="B15" s="18">
         <f>A15-$B$10</f>
@@ -3795,7 +3725,7 @@
         <v/>
       </c>
       <c r="H15" s="16">
-        <f>($B$11)*(IF(B15&lt;=0,0,IF(B15&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1))+(B15-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B15&lt;=0,0,IF(B15&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1))+(B15-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B15,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I15" s="16">
@@ -3809,7 +3739,7 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="n">
-        <v>35.18</v>
+        <v>34.98</v>
       </c>
       <c r="B16" s="18">
         <f>A16-$B$10</f>
@@ -3836,7 +3766,7 @@
         <v/>
       </c>
       <c r="H16" s="16">
-        <f>($B$11)*(IF(B16&lt;=0,0,IF(B16&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1))+(B16-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B16&lt;=0,0,IF(B16&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1))+(B16-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B16,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I16" s="16">
@@ -3850,7 +3780,7 @@
     </row>
     <row r="17">
       <c r="A17" s="18" t="n">
-        <v>35.28</v>
+        <v>35.08</v>
       </c>
       <c r="B17" s="18">
         <f>A17-$B$10</f>
@@ -3877,7 +3807,7 @@
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>($B$11)*(IF(B17&lt;=0,0,IF(B17&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1))+(B17-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B17&lt;=0,0,IF(B17&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1))+(B17-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B17,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I17" s="16">
@@ -3891,7 +3821,7 @@
     </row>
     <row r="18">
       <c r="A18" s="18" t="n">
-        <v>35.38</v>
+        <v>35.18</v>
       </c>
       <c r="B18" s="18">
         <f>A18-$B$10</f>
@@ -3918,7 +3848,7 @@
         <v/>
       </c>
       <c r="H18" s="16">
-        <f>($B$11)*(IF(B18&lt;=0,0,IF(B18&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1))+(B18-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B18&lt;=0,0,IF(B18&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1))+(B18-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B18,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I18" s="16">
@@ -3932,7 +3862,7 @@
     </row>
     <row r="19">
       <c r="A19" s="18" t="n">
-        <v>35.48</v>
+        <v>35.28</v>
       </c>
       <c r="B19" s="18">
         <f>A19-$B$10</f>
@@ -3959,7 +3889,7 @@
         <v/>
       </c>
       <c r="H19" s="16">
-        <f>($B$11)*(IF(B19&lt;=0,0,IF(B19&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1))+(B19-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B19&lt;=0,0,IF(B19&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1))+(B19-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B19,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I19" s="16">
@@ -3973,7 +3903,7 @@
     </row>
     <row r="20">
       <c r="A20" s="18" t="n">
-        <v>35.58</v>
+        <v>35.38</v>
       </c>
       <c r="B20" s="18">
         <f>A20-$B$10</f>
@@ -4000,7 +3930,7 @@
         <v/>
       </c>
       <c r="H20" s="16">
-        <f>($B$11)*(IF(B20&lt;=0,0,IF(B20&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1))+(B20-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B20&lt;=0,0,IF(B20&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1))+(B20-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B20,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I20" s="16">
@@ -4014,7 +3944,7 @@
     </row>
     <row r="21">
       <c r="A21" s="18" t="n">
-        <v>35.68</v>
+        <v>35.48</v>
       </c>
       <c r="B21" s="18">
         <f>A21-$B$10</f>
@@ -4041,7 +3971,7 @@
         <v/>
       </c>
       <c r="H21" s="16">
-        <f>($B$11)*(IF(B21&lt;=0,0,IF(B21&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1))+(B21-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B21&lt;=0,0,IF(B21&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1))+(B21-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B21,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I21" s="16">
@@ -4055,7 +3985,7 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="n">
-        <v>35.78</v>
+        <v>35.58</v>
       </c>
       <c r="B22" s="18">
         <f>A22-$B$10</f>
@@ -4082,7 +4012,7 @@
         <v/>
       </c>
       <c r="H22" s="16">
-        <f>($B$11)*(IF(B22&lt;=0,0,IF(B22&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1))+(B22-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B22&lt;=0,0,IF(B22&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1))+(B22-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B22,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I22" s="16">
@@ -4096,7 +4026,7 @@
     </row>
     <row r="23">
       <c r="A23" s="18" t="n">
-        <v>35.88</v>
+        <v>35.68</v>
       </c>
       <c r="B23" s="18">
         <f>A23-$B$10</f>
@@ -4123,7 +4053,7 @@
         <v/>
       </c>
       <c r="H23" s="16">
-        <f>($B$11)*(IF(B23&lt;=0,0,IF(B23&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1))+(B23-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B23&lt;=0,0,IF(B23&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1))+(B23-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B23,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I23" s="16">
@@ -4137,7 +4067,7 @@
     </row>
     <row r="24">
       <c r="A24" s="18" t="n">
-        <v>35.98</v>
+        <v>35.78</v>
       </c>
       <c r="B24" s="18">
         <f>A24-$B$10</f>
@@ -4164,7 +4094,7 @@
         <v/>
       </c>
       <c r="H24" s="16">
-        <f>($B$11)*(IF(B24&lt;=0,0,IF(B24&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1))+(B24-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B24&lt;=0,0,IF(B24&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1))+(B24-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B24,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I24" s="16">
@@ -4178,7 +4108,7 @@
     </row>
     <row r="25">
       <c r="A25" s="18" t="n">
-        <v>36.08</v>
+        <v>35.88</v>
       </c>
       <c r="B25" s="18">
         <f>A25-$B$10</f>
@@ -4205,7 +4135,7 @@
         <v/>
       </c>
       <c r="H25" s="16">
-        <f>($B$11)*(IF(B25&lt;=0,0,IF(B25&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1))+(B25-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B25&lt;=0,0,IF(B25&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1))+(B25-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B25,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I25" s="16">
@@ -4219,7 +4149,7 @@
     </row>
     <row r="26">
       <c r="A26" s="18" t="n">
-        <v>36.18</v>
+        <v>35.98</v>
       </c>
       <c r="B26" s="18">
         <f>A26-$B$10</f>
@@ -4246,7 +4176,7 @@
         <v/>
       </c>
       <c r="H26" s="16">
-        <f>($B$11)*(IF(B26&lt;=0,0,IF(B26&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1))+(B26-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B26&lt;=0,0,IF(B26&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1))+(B26-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B26,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I26" s="16">
@@ -4260,7 +4190,7 @@
     </row>
     <row r="27">
       <c r="A27" s="18" t="n">
-        <v>36.28</v>
+        <v>36.08</v>
       </c>
       <c r="B27" s="18">
         <f>A27-$B$10</f>
@@ -4287,7 +4217,7 @@
         <v/>
       </c>
       <c r="H27" s="16">
-        <f>($B$11)*(IF(B27&lt;=0,0,IF(B27&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1))+(B27-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B27&lt;=0,0,IF(B27&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1))+(B27-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B27,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I27" s="16">
@@ -4301,7 +4231,7 @@
     </row>
     <row r="28">
       <c r="A28" s="18" t="n">
-        <v>36.38</v>
+        <v>36.18</v>
       </c>
       <c r="B28" s="18">
         <f>A28-$B$10</f>
@@ -4328,7 +4258,7 @@
         <v/>
       </c>
       <c r="H28" s="16">
-        <f>($B$11)*(IF(B28&lt;=0,0,IF(B28&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1))+(B28-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B28&lt;=0,0,IF(B28&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1))+(B28-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B28,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I28" s="16">
@@ -4342,7 +4272,7 @@
     </row>
     <row r="29">
       <c r="A29" s="18" t="n">
-        <v>36.48</v>
+        <v>36.28</v>
       </c>
       <c r="B29" s="18">
         <f>A29-$B$10</f>
@@ -4369,7 +4299,7 @@
         <v/>
       </c>
       <c r="H29" s="16">
-        <f>($B$11)*(IF(B29&lt;=0,0,IF(B29&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1))+(B29-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B29&lt;=0,0,IF(B29&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1))+(B29-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B29,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I29" s="16">
@@ -4383,7 +4313,7 @@
     </row>
     <row r="30">
       <c r="A30" s="18" t="n">
-        <v>36.58</v>
+        <v>36.38</v>
       </c>
       <c r="B30" s="18">
         <f>A30-$B$10</f>
@@ -4410,7 +4340,7 @@
         <v/>
       </c>
       <c r="H30" s="16">
-        <f>($B$11)*(IF(B30&lt;=0,0,IF(B30&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1))+(B30-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B30&lt;=0,0,IF(B30&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1))+(B30-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B30,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I30" s="16">
@@ -4424,7 +4354,7 @@
     </row>
     <row r="31">
       <c r="A31" s="18" t="n">
-        <v>36.68</v>
+        <v>36.48</v>
       </c>
       <c r="B31" s="18">
         <f>A31-$B$10</f>
@@ -4451,7 +4381,7 @@
         <v/>
       </c>
       <c r="H31" s="16">
-        <f>($B$11)*(IF(B31&lt;=0,0,IF(B31&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1))+(B31-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B31&lt;=0,0,IF(B31&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1))+(B31-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B31,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I31" s="16">
@@ -4465,7 +4395,7 @@
     </row>
     <row r="32">
       <c r="A32" s="18" t="n">
-        <v>36.78</v>
+        <v>36.58</v>
       </c>
       <c r="B32" s="18">
         <f>A32-$B$10</f>
@@ -4492,7 +4422,7 @@
         <v/>
       </c>
       <c r="H32" s="16">
-        <f>($B$11)*(IF(B32&lt;=0,0,IF(B32&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1))+(B32-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B32&lt;=0,0,IF(B32&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1))+(B32-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B32,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I32" s="16">
@@ -4506,7 +4436,7 @@
     </row>
     <row r="33">
       <c r="A33" s="18" t="n">
-        <v>36.88</v>
+        <v>36.68</v>
       </c>
       <c r="B33" s="18">
         <f>A33-$B$10</f>
@@ -4533,7 +4463,7 @@
         <v/>
       </c>
       <c r="H33" s="16">
-        <f>($B$11)*(IF(B33&lt;=0,0,IF(B33&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1))+(B33-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B33&lt;=0,0,IF(B33&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1))+(B33-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B33,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I33" s="16">
@@ -4547,7 +4477,7 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="n">
-        <v>36.98</v>
+        <v>36.78</v>
       </c>
       <c r="B34" s="18">
         <f>A34-$B$10</f>
@@ -4574,7 +4504,7 @@
         <v/>
       </c>
       <c r="H34" s="16">
-        <f>($B$11)*(IF(B34&lt;=0,0,IF(B34&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1))+(B34-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B34&lt;=0,0,IF(B34&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1))+(B34-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B34,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I34" s="16">
@@ -4588,7 +4518,7 @@
     </row>
     <row r="35">
       <c r="A35" s="18" t="n">
-        <v>37.08</v>
+        <v>36.88</v>
       </c>
       <c r="B35" s="18">
         <f>A35-$B$10</f>
@@ -4615,7 +4545,7 @@
         <v/>
       </c>
       <c r="H35" s="16">
-        <f>($B$11)*(IF(B35&lt;=0,0,IF(B35&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1))+(B35-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B35&lt;=0,0,IF(B35&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1))+(B35-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B35,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I35" s="16">
@@ -4629,7 +4559,7 @@
     </row>
     <row r="36">
       <c r="A36" s="18" t="n">
-        <v>37.18</v>
+        <v>36.98</v>
       </c>
       <c r="B36" s="18">
         <f>A36-$B$10</f>
@@ -4656,7 +4586,7 @@
         <v/>
       </c>
       <c r="H36" s="16">
-        <f>($B$11)*(IF(B36&lt;=0,0,IF(B36&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1))+(B36-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B36&lt;=0,0,IF(B36&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1))+(B36-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B36,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I36" s="16">
@@ -4670,7 +4600,7 @@
     </row>
     <row r="37">
       <c r="A37" s="18" t="n">
-        <v>37.28</v>
+        <v>37.08</v>
       </c>
       <c r="B37" s="18">
         <f>A37-$B$10</f>
@@ -4697,7 +4627,7 @@
         <v/>
       </c>
       <c r="H37" s="16">
-        <f>($B$11)*(IF(B37&lt;=0,0,IF(B37&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1))+(B37-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B37&lt;=0,0,IF(B37&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1))+(B37-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B37,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I37" s="16">
@@ -4711,7 +4641,7 @@
     </row>
     <row r="38">
       <c r="A38" s="18" t="n">
-        <v>37.38</v>
+        <v>37.18</v>
       </c>
       <c r="B38" s="18">
         <f>A38-$B$10</f>
@@ -4738,7 +4668,7 @@
         <v/>
       </c>
       <c r="H38" s="16">
-        <f>($B$11)*(IF(B38&lt;=0,0,IF(B38&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1))+(B38-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B38&lt;=0,0,IF(B38&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1))+(B38-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B38,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I38" s="16">
@@ -4752,7 +4682,7 @@
     </row>
     <row r="39">
       <c r="A39" s="18" t="n">
-        <v>37.48</v>
+        <v>37.28</v>
       </c>
       <c r="B39" s="18">
         <f>A39-$B$10</f>
@@ -4779,7 +4709,7 @@
         <v/>
       </c>
       <c r="H39" s="16">
-        <f>($B$11)*(IF(B39&lt;=0,0,IF(B39&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1))+(B39-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B39&lt;=0,0,IF(B39&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1))+(B39-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B39,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I39" s="16">
@@ -4793,7 +4723,7 @@
     </row>
     <row r="40">
       <c r="A40" s="18" t="n">
-        <v>37.58</v>
+        <v>37.38</v>
       </c>
       <c r="B40" s="18">
         <f>A40-$B$10</f>
@@ -4820,7 +4750,7 @@
         <v/>
       </c>
       <c r="H40" s="16">
-        <f>($B$11)*(IF(B40&lt;=0,0,IF(B40&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1))+(B40-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B40&lt;=0,0,IF(B40&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1))+(B40-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B40,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I40" s="16">
@@ -4834,7 +4764,7 @@
     </row>
     <row r="41">
       <c r="A41" s="18" t="n">
-        <v>37.68</v>
+        <v>37.48</v>
       </c>
       <c r="B41" s="18">
         <f>A41-$B$10</f>
@@ -4861,7 +4791,7 @@
         <v/>
       </c>
       <c r="H41" s="16">
-        <f>($B$11)*(IF(B41&lt;=0,0,IF(B41&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1))+(B41-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B41&lt;=0,0,IF(B41&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1))+(B41-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B41,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I41" s="16">
@@ -4875,7 +4805,7 @@
     </row>
     <row r="42">
       <c r="A42" s="18" t="n">
-        <v>37.78</v>
+        <v>37.58</v>
       </c>
       <c r="B42" s="18">
         <f>A42-$B$10</f>
@@ -4902,7 +4832,7 @@
         <v/>
       </c>
       <c r="H42" s="16">
-        <f>($B$11)*(IF(B42&lt;=0,0,IF(B42&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1))+(B42-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B42&lt;=0,0,IF(B42&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1))+(B42-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B42,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I42" s="16">
@@ -4916,7 +4846,7 @@
     </row>
     <row r="43">
       <c r="A43" s="18" t="n">
-        <v>37.88</v>
+        <v>37.68</v>
       </c>
       <c r="B43" s="18">
         <f>A43-$B$10</f>
@@ -4943,7 +4873,7 @@
         <v/>
       </c>
       <c r="H43" s="16">
-        <f>($B$11)*(IF(B43&lt;=0,0,IF(B43&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1))+(B43-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B43&lt;=0,0,IF(B43&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1))+(B43-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B43,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I43" s="16">
@@ -4957,7 +4887,7 @@
     </row>
     <row r="44">
       <c r="A44" s="18" t="n">
-        <v>37.98</v>
+        <v>37.78</v>
       </c>
       <c r="B44" s="18">
         <f>A44-$B$10</f>
@@ -4984,7 +4914,7 @@
         <v/>
       </c>
       <c r="H44" s="16">
-        <f>($B$11)*(IF(B44&lt;=0,0,IF(B44&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1))+(B44-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B44&lt;=0,0,IF(B44&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1))+(B44-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B44,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I44" s="16">
@@ -4998,7 +4928,7 @@
     </row>
     <row r="45">
       <c r="A45" s="18" t="n">
-        <v>38.08</v>
+        <v>37.88</v>
       </c>
       <c r="B45" s="18">
         <f>A45-$B$10</f>
@@ -5025,7 +4955,7 @@
         <v/>
       </c>
       <c r="H45" s="16">
-        <f>($B$11)*(IF(B45&lt;=0,0,IF(B45&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1))+(B45-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B45&lt;=0,0,IF(B45&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1))+(B45-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B45,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I45" s="16">
@@ -5039,7 +4969,7 @@
     </row>
     <row r="46">
       <c r="A46" s="18" t="n">
-        <v>38.18</v>
+        <v>37.98</v>
       </c>
       <c r="B46" s="18">
         <f>A46-$B$10</f>
@@ -5066,7 +4996,7 @@
         <v/>
       </c>
       <c r="H46" s="16">
-        <f>($B$11)*(IF(B46&lt;=0,0,IF(B46&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1))+(B46-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B46&lt;=0,0,IF(B46&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1))+(B46-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B46,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I46" s="16">
@@ -5080,7 +5010,7 @@
     </row>
     <row r="47">
       <c r="A47" s="18" t="n">
-        <v>38.28</v>
+        <v>38.08</v>
       </c>
       <c r="B47" s="18">
         <f>A47-$B$10</f>
@@ -5107,7 +5037,7 @@
         <v/>
       </c>
       <c r="H47" s="16">
-        <f>($B$11)*(IF(B47&lt;=0,0,IF(B47&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1))+(B47-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B47&lt;=0,0,IF(B47&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1))+(B47-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B47,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I47" s="16">
@@ -5121,7 +5051,7 @@
     </row>
     <row r="48">
       <c r="A48" s="18" t="n">
-        <v>38.38</v>
+        <v>38.18</v>
       </c>
       <c r="B48" s="18">
         <f>A48-$B$10</f>
@@ -5148,7 +5078,7 @@
         <v/>
       </c>
       <c r="H48" s="16">
-        <f>($B$11)*(IF(B48&lt;=0,0,IF(B48&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1))+(B48-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B48&lt;=0,0,IF(B48&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1))+(B48-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B48,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I48" s="16">
@@ -5162,7 +5092,7 @@
     </row>
     <row r="49">
       <c r="A49" s="18" t="n">
-        <v>38.48</v>
+        <v>38.28</v>
       </c>
       <c r="B49" s="18">
         <f>A49-$B$10</f>
@@ -5189,7 +5119,7 @@
         <v/>
       </c>
       <c r="H49" s="16">
-        <f>($B$11)*(IF(B49&lt;=0,0,IF(B49&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1))+(B49-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B49&lt;=0,0,IF(B49&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1))+(B49-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B49,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I49" s="16">
@@ -5203,7 +5133,7 @@
     </row>
     <row r="50">
       <c r="A50" s="18" t="n">
-        <v>38.58</v>
+        <v>38.38</v>
       </c>
       <c r="B50" s="18">
         <f>A50-$B$10</f>
@@ -5230,7 +5160,7 @@
         <v/>
       </c>
       <c r="H50" s="16">
-        <f>($B$11)*(IF(B50&lt;=0,0,IF(B50&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1))+(B50-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B50&lt;=0,0,IF(B50&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1))+(B50-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B50,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I50" s="16">
@@ -5244,7 +5174,7 @@
     </row>
     <row r="51">
       <c r="A51" s="18" t="n">
-        <v>38.68</v>
+        <v>38.48</v>
       </c>
       <c r="B51" s="18">
         <f>A51-$B$10</f>
@@ -5271,7 +5201,7 @@
         <v/>
       </c>
       <c r="H51" s="16">
-        <f>($B$11)*(IF(B51&lt;=0,0,IF(B51&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1))+(B51-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B51&lt;=0,0,IF(B51&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1))+(B51-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B51,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I51" s="16">
@@ -5285,7 +5215,7 @@
     </row>
     <row r="52">
       <c r="A52" s="18" t="n">
-        <v>38.78</v>
+        <v>38.58</v>
       </c>
       <c r="B52" s="18">
         <f>A52-$B$10</f>
@@ -5312,7 +5242,7 @@
         <v/>
       </c>
       <c r="H52" s="16">
-        <f>($B$11)*(IF(B52&lt;=0,0,IF(B52&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1))+(B52-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B52&lt;=0,0,IF(B52&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1))+(B52-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B52,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I52" s="16">
@@ -5326,7 +5256,7 @@
     </row>
     <row r="53">
       <c r="A53" s="18" t="n">
-        <v>38.88</v>
+        <v>38.68</v>
       </c>
       <c r="B53" s="18">
         <f>A53-$B$10</f>
@@ -5353,7 +5283,7 @@
         <v/>
       </c>
       <c r="H53" s="16">
-        <f>($B$11)*(IF(B53&lt;=0,0,IF(B53&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1))+(B53-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B53&lt;=0,0,IF(B53&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1))+(B53-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B53,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I53" s="16">
@@ -5367,7 +5297,7 @@
     </row>
     <row r="54">
       <c r="A54" s="18" t="n">
-        <v>38.98</v>
+        <v>38.78</v>
       </c>
       <c r="B54" s="18">
         <f>A54-$B$10</f>
@@ -5394,7 +5324,7 @@
         <v/>
       </c>
       <c r="H54" s="16">
-        <f>($B$11)*(IF(B54&lt;=0,0,IF(B54&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1))+(B54-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B54&lt;=0,0,IF(B54&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1))+(B54-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B54,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I54" s="16">
@@ -5408,7 +5338,7 @@
     </row>
     <row r="55">
       <c r="A55" s="18" t="n">
-        <v>39.08</v>
+        <v>38.88</v>
       </c>
       <c r="B55" s="18">
         <f>A55-$B$10</f>
@@ -5435,7 +5365,7 @@
         <v/>
       </c>
       <c r="H55" s="16">
-        <f>($B$11)*(IF(B55&lt;=0,0,IF(B55&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1))+(B55-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B55&lt;=0,0,IF(B55&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1))+(B55-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B55,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I55" s="16">
@@ -5449,7 +5379,7 @@
     </row>
     <row r="56">
       <c r="A56" s="18" t="n">
-        <v>39.18</v>
+        <v>38.98</v>
       </c>
       <c r="B56" s="18">
         <f>A56-$B$10</f>
@@ -5476,7 +5406,7 @@
         <v/>
       </c>
       <c r="H56" s="16">
-        <f>($B$11)*(IF(B56&lt;=0,0,IF(B56&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1))+(B56-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B56&lt;=0,0,IF(B56&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1))+(B56-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B56,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I56" s="16">
@@ -5490,7 +5420,7 @@
     </row>
     <row r="57">
       <c r="A57" s="18" t="n">
-        <v>39.28</v>
+        <v>39.08</v>
       </c>
       <c r="B57" s="18">
         <f>A57-$B$10</f>
@@ -5517,7 +5447,7 @@
         <v/>
       </c>
       <c r="H57" s="16">
-        <f>($B$11)*(IF(B57&lt;=0,0,IF(B57&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1))+(B57-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B57&lt;=0,0,IF(B57&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1))+(B57-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B57,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I57" s="16">
@@ -5531,7 +5461,7 @@
     </row>
     <row r="58">
       <c r="A58" s="18" t="n">
-        <v>39.38</v>
+        <v>39.18</v>
       </c>
       <c r="B58" s="18">
         <f>A58-$B$10</f>
@@ -5558,7 +5488,7 @@
         <v/>
       </c>
       <c r="H58" s="16">
-        <f>($B$11)*(IF(B58&lt;=0,0,IF(B58&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1))+(B58-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B58&lt;=0,0,IF(B58&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1))+(B58-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B58,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I58" s="16">
@@ -5572,7 +5502,7 @@
     </row>
     <row r="59">
       <c r="A59" s="18" t="n">
-        <v>39.48</v>
+        <v>39.28</v>
       </c>
       <c r="B59" s="18">
         <f>A59-$B$10</f>
@@ -5599,7 +5529,7 @@
         <v/>
       </c>
       <c r="H59" s="16">
-        <f>($B$11)*(IF(B59&lt;=0,0,IF(B59&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1))+(B59-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B59&lt;=0,0,IF(B59&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1))+(B59-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B59,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I59" s="16">
@@ -5613,7 +5543,7 @@
     </row>
     <row r="60">
       <c r="A60" s="18" t="n">
-        <v>39.58</v>
+        <v>39.38</v>
       </c>
       <c r="B60" s="18">
         <f>A60-$B$10</f>
@@ -5640,7 +5570,7 @@
         <v/>
       </c>
       <c r="H60" s="16">
-        <f>($B$11)*(IF(B60&lt;=0,0,IF(B60&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1))+(B60-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B60&lt;=0,0,IF(B60&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1))+(B60-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I60" s="16">
@@ -5654,7 +5584,7 @@
     </row>
     <row r="61">
       <c r="A61" s="18" t="n">
-        <v>39.68</v>
+        <v>39.48</v>
       </c>
       <c r="B61" s="18">
         <f>A61-$B$10</f>
@@ -5681,7 +5611,7 @@
         <v/>
       </c>
       <c r="H61" s="16">
-        <f>($B$11)*(IF(B61&lt;=0,0,IF(B61&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1))+(B61-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B61&lt;=0,0,IF(B61&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1))+(B61-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I61" s="16">
@@ -5695,7 +5625,7 @@
     </row>
     <row r="62">
       <c r="A62" s="18" t="n">
-        <v>39.78</v>
+        <v>39.58</v>
       </c>
       <c r="B62" s="18">
         <f>A62-$B$10</f>
@@ -5722,7 +5652,7 @@
         <v/>
       </c>
       <c r="H62" s="16">
-        <f>($B$11)*(IF(B62&lt;=0,0,IF(B62&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1))+(B62-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B62&lt;=0,0,IF(B62&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1))+(B62-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I62" s="16">
@@ -5736,7 +5666,7 @@
     </row>
     <row r="63">
       <c r="A63" s="18" t="n">
-        <v>39.88</v>
+        <v>39.68</v>
       </c>
       <c r="B63" s="18">
         <f>A63-$B$10</f>
@@ -5763,7 +5693,7 @@
         <v/>
       </c>
       <c r="H63" s="16">
-        <f>($B$11)*(IF(B63&lt;=0,0,IF(B63&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1))+(B63-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B63&lt;=0,0,IF(B63&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1))+(B63-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I63" s="16">
@@ -5777,7 +5707,7 @@
     </row>
     <row r="64">
       <c r="A64" s="18" t="n">
-        <v>39.98</v>
+        <v>39.78</v>
       </c>
       <c r="B64" s="18">
         <f>A64-$B$10</f>
@@ -5804,7 +5734,7 @@
         <v/>
       </c>
       <c r="H64" s="16">
-        <f>($B$11)*(IF(B64&lt;=0,0,IF(B64&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1))+(B64-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1))))))</f>
+        <f>MIN($B$12,($B$11)*(IF(B64&lt;=0,0,IF(B64&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1))+(B64-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
         <v/>
       </c>
       <c r="I64" s="16">
@@ -5813,6 +5743,88 @@
       </c>
       <c r="J64" s="8">
         <f>H64+I64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="n">
+        <v>39.88</v>
+      </c>
+      <c r="B65" s="18">
+        <f>A65-$B$10</f>
+        <v/>
+      </c>
+      <c r="C65" s="18">
+        <f>MAX(0,A65-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D65" s="16">
+        <f>IF(C65&lt;=0,0,($B$5+$B$7*C65)*C65)</f>
+        <v/>
+      </c>
+      <c r="E65" s="15">
+        <f>D65*$B$9</f>
+        <v/>
+      </c>
+      <c r="F65" s="15">
+        <f>IF(A65&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A65&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1))+(A65-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G65" s="12">
+        <f>E65+F65</f>
+        <v/>
+      </c>
+      <c r="H65" s="16">
+        <f>MIN($B$12,($B$11)*(IF(B65&lt;=0,0,IF(B65&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B65,Courbe_QH_1200!$A$20:$A$80,1))+(B65-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B65,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B65,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B65,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B65,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B65,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
+        <v/>
+      </c>
+      <c r="I65" s="16">
+        <f>IF(C65&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D65*IF(($B$5+2*C65*SQRT(1+$B$7^2))&lt;=0,0,((D65/($B$5+2*C65*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J65" s="8">
+        <f>H65+I65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="B66" s="18">
+        <f>A66-$B$10</f>
+        <v/>
+      </c>
+      <c r="C66" s="18">
+        <f>MAX(0,A66-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D66" s="16">
+        <f>IF(C66&lt;=0,0,($B$5+$B$7*C66)*C66)</f>
+        <v/>
+      </c>
+      <c r="E66" s="15">
+        <f>D66*$B$9</f>
+        <v/>
+      </c>
+      <c r="F66" s="15">
+        <f>IF(A66&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A66&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1))+(A66-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G66" s="12">
+        <f>E66+F66</f>
+        <v/>
+      </c>
+      <c r="H66" s="16">
+        <f>MIN($B$12,($B$11)*(IF(B66&lt;=0,0,IF(B66&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B66,Courbe_QH_1200!$A$20:$A$80,1))+(B66-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B66,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B66,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B66,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B66,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B66,Courbe_QH_1200!$A$20:$A$80,1)))))))</f>
+        <v/>
+      </c>
+      <c r="I66" s="16">
+        <f>IF(C66&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D66*IF(($B$5+2*C66*SQRT(1+$B$7^2))&lt;=0,0,((D66/($B$5+2*C66*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J66" s="8">
+        <f>H66+I66</f>
         <v/>
       </c>
     </row>
@@ -6058,11 +6070,11 @@
         <v/>
       </c>
       <c r="C16" s="16">
-        <f>IF(F15&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F15&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F15,Compose!$G$13:$G$64,1))+(F15-INDEX(Compose!$G$13:$G$64,MATCH(F15,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F15,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F15,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F15,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F15,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F15&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F15&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F15,Compose!$G$15:$G$66,1))+(F15-INDEX(Compose!$G$15:$G$66,MATCH(F15,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F15,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F15,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F15,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F15,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>IF(F15&lt;=0.01,MIN(0.5*(B15+B16),$B$4),IF(C16&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C16&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C16,Compose!$A$13:$A$64,1))+(C16-INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C16,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C16,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F15&lt;=0.01,MIN(0.5*(B15+B16),$B$4),IF(C16&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C16&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C16,Compose!$A$15:$A$66,1))+(C16-INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C16,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C16,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E16" s="15">
@@ -6074,11 +6086,11 @@
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IF(C16&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C16&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C16,Compose!$A$13:$A$64,1))+(C16-INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C16,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C16,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C16&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C16&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C16,Compose!$A$15:$A$66,1))+(C16-INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C16,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C16,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H16" s="16">
-        <f>IF(C16&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C16&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C16,Compose!$A$13:$A$64,1))+(C16-INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C16,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C16,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C16,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C16&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C16&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C16,Compose!$A$15:$A$66,1))+(C16-INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C16,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C16,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C16,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I16" s="20">
@@ -6100,11 +6112,11 @@
         <v/>
       </c>
       <c r="C17" s="16">
-        <f>IF(F16&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F16&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F16,Compose!$G$13:$G$64,1))+(F16-INDEX(Compose!$G$13:$G$64,MATCH(F16,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F16,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F16,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F16,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F16,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F16&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F16&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F16,Compose!$G$15:$G$66,1))+(F16-INDEX(Compose!$G$15:$G$66,MATCH(F16,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F16,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F16,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F16,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F16,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>IF(F16&lt;=0.01,MIN(0.5*(B16+B17),$B$4),IF(C17&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C17&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C17,Compose!$A$13:$A$64,1))+(C17-INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C17,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C17,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F16&lt;=0.01,MIN(0.5*(B16+B17),$B$4),IF(C17&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C17&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C17,Compose!$A$15:$A$66,1))+(C17-INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C17,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C17,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E17" s="15">
@@ -6116,11 +6128,11 @@
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>IF(C17&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C17&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C17,Compose!$A$13:$A$64,1))+(C17-INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C17,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C17,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C17&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C17&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C17,Compose!$A$15:$A$66,1))+(C17-INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C17,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C17,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>IF(C17&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C17&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C17,Compose!$A$13:$A$64,1))+(C17-INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C17,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C17,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C17,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C17&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C17&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C17,Compose!$A$15:$A$66,1))+(C17-INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C17,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C17,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C17,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I17" s="20">
@@ -6142,11 +6154,11 @@
         <v/>
       </c>
       <c r="C18" s="16">
-        <f>IF(F17&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F17&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F17,Compose!$G$13:$G$64,1))+(F17-INDEX(Compose!$G$13:$G$64,MATCH(F17,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F17,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F17,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F17,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F17,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F17&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F17&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F17,Compose!$G$15:$G$66,1))+(F17-INDEX(Compose!$G$15:$G$66,MATCH(F17,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F17,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F17,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F17,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F17,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D18" s="16">
-        <f>IF(F17&lt;=0.01,MIN(0.5*(B17+B18),$B$4),IF(C18&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C18&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C18,Compose!$A$13:$A$64,1))+(C18-INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C18,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C18,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F17&lt;=0.01,MIN(0.5*(B17+B18),$B$4),IF(C18&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C18&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C18,Compose!$A$15:$A$66,1))+(C18-INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C18,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C18,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E18" s="15">
@@ -6158,11 +6170,11 @@
         <v/>
       </c>
       <c r="G18" s="16">
-        <f>IF(C18&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C18&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C18,Compose!$A$13:$A$64,1))+(C18-INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C18,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C18,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C18&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C18&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C18,Compose!$A$15:$A$66,1))+(C18-INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C18,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C18,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H18" s="16">
-        <f>IF(C18&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C18&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C18,Compose!$A$13:$A$64,1))+(C18-INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C18,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C18,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C18,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C18&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C18&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C18,Compose!$A$15:$A$66,1))+(C18-INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C18,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C18,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C18,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I18" s="20">
@@ -6184,11 +6196,11 @@
         <v/>
       </c>
       <c r="C19" s="16">
-        <f>IF(F18&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F18&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F18,Compose!$G$13:$G$64,1))+(F18-INDEX(Compose!$G$13:$G$64,MATCH(F18,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F18,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F18,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F18,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F18,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F18&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F18&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F18,Compose!$G$15:$G$66,1))+(F18-INDEX(Compose!$G$15:$G$66,MATCH(F18,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F18,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F18,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F18,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F18,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D19" s="16">
-        <f>IF(F18&lt;=0.01,MIN(0.5*(B18+B19),$B$4),IF(C19&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C19&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C19,Compose!$A$13:$A$64,1))+(C19-INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C19,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C19,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F18&lt;=0.01,MIN(0.5*(B18+B19),$B$4),IF(C19&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C19&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C19,Compose!$A$15:$A$66,1))+(C19-INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C19,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C19,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E19" s="15">
@@ -6200,11 +6212,11 @@
         <v/>
       </c>
       <c r="G19" s="16">
-        <f>IF(C19&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C19&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C19,Compose!$A$13:$A$64,1))+(C19-INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C19,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C19,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C19&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C19&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C19,Compose!$A$15:$A$66,1))+(C19-INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C19,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C19,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H19" s="16">
-        <f>IF(C19&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C19&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C19,Compose!$A$13:$A$64,1))+(C19-INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C19,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C19,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C19,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C19&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C19&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C19,Compose!$A$15:$A$66,1))+(C19-INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C19,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C19,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C19,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I19" s="20">
@@ -6226,11 +6238,11 @@
         <v/>
       </c>
       <c r="C20" s="16">
-        <f>IF(F19&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F19&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F19,Compose!$G$13:$G$64,1))+(F19-INDEX(Compose!$G$13:$G$64,MATCH(F19,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F19,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F19,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F19,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F19,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F19&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F19&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F19,Compose!$G$15:$G$66,1))+(F19-INDEX(Compose!$G$15:$G$66,MATCH(F19,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F19,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F19,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F19,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F19,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D20" s="16">
-        <f>IF(F19&lt;=0.01,MIN(0.5*(B19+B20),$B$4),IF(C20&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C20&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C20,Compose!$A$13:$A$64,1))+(C20-INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C20,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C20,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F19&lt;=0.01,MIN(0.5*(B19+B20),$B$4),IF(C20&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C20&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C20,Compose!$A$15:$A$66,1))+(C20-INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C20,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C20,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E20" s="15">
@@ -6242,11 +6254,11 @@
         <v/>
       </c>
       <c r="G20" s="16">
-        <f>IF(C20&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C20&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C20,Compose!$A$13:$A$64,1))+(C20-INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C20,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C20,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C20&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C20&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C20,Compose!$A$15:$A$66,1))+(C20-INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C20,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C20,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H20" s="16">
-        <f>IF(C20&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C20&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C20,Compose!$A$13:$A$64,1))+(C20-INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C20,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C20,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C20,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C20&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C20&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C20,Compose!$A$15:$A$66,1))+(C20-INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C20,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C20,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C20,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I20" s="20">
@@ -6268,11 +6280,11 @@
         <v/>
       </c>
       <c r="C21" s="16">
-        <f>IF(F20&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F20&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F20,Compose!$G$13:$G$64,1))+(F20-INDEX(Compose!$G$13:$G$64,MATCH(F20,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F20,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F20,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F20,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F20,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F20&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F20&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F20,Compose!$G$15:$G$66,1))+(F20-INDEX(Compose!$G$15:$G$66,MATCH(F20,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F20,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F20,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F20,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F20,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D21" s="16">
-        <f>IF(F20&lt;=0.01,MIN(0.5*(B20+B21),$B$4),IF(C21&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C21&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C21,Compose!$A$13:$A$64,1))+(C21-INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C21,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C21,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F20&lt;=0.01,MIN(0.5*(B20+B21),$B$4),IF(C21&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C21&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C21,Compose!$A$15:$A$66,1))+(C21-INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C21,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C21,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E21" s="15">
@@ -6284,11 +6296,11 @@
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>IF(C21&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C21&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C21,Compose!$A$13:$A$64,1))+(C21-INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C21,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C21,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C21&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C21&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C21,Compose!$A$15:$A$66,1))+(C21-INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C21,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C21,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H21" s="16">
-        <f>IF(C21&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C21&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C21,Compose!$A$13:$A$64,1))+(C21-INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C21,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C21,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C21,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C21&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C21&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C21,Compose!$A$15:$A$66,1))+(C21-INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C21,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C21,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C21,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I21" s="20">
@@ -6310,11 +6322,11 @@
         <v/>
       </c>
       <c r="C22" s="16">
-        <f>IF(F21&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F21&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F21,Compose!$G$13:$G$64,1))+(F21-INDEX(Compose!$G$13:$G$64,MATCH(F21,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F21,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F21,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F21,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F21,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F21&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F21&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F21,Compose!$G$15:$G$66,1))+(F21-INDEX(Compose!$G$15:$G$66,MATCH(F21,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F21,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F21,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F21,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F21,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D22" s="16">
-        <f>IF(F21&lt;=0.01,MIN(0.5*(B21+B22),$B$4),IF(C22&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C22&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C22,Compose!$A$13:$A$64,1))+(C22-INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C22,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C22,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F21&lt;=0.01,MIN(0.5*(B21+B22),$B$4),IF(C22&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C22&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C22,Compose!$A$15:$A$66,1))+(C22-INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C22,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C22,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E22" s="15">
@@ -6326,11 +6338,11 @@
         <v/>
       </c>
       <c r="G22" s="16">
-        <f>IF(C22&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C22&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C22,Compose!$A$13:$A$64,1))+(C22-INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C22,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C22,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C22&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C22&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C22,Compose!$A$15:$A$66,1))+(C22-INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C22,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C22,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H22" s="16">
-        <f>IF(C22&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C22&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C22,Compose!$A$13:$A$64,1))+(C22-INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C22,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C22,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C22,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C22&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C22&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C22,Compose!$A$15:$A$66,1))+(C22-INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C22,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C22,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C22,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I22" s="20">
@@ -6352,11 +6364,11 @@
         <v/>
       </c>
       <c r="C23" s="16">
-        <f>IF(F22&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F22&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F22,Compose!$G$13:$G$64,1))+(F22-INDEX(Compose!$G$13:$G$64,MATCH(F22,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F22,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F22,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F22,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F22,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F22&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F22&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F22,Compose!$G$15:$G$66,1))+(F22-INDEX(Compose!$G$15:$G$66,MATCH(F22,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F22,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F22,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F22,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F22,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D23" s="16">
-        <f>IF(F22&lt;=0.01,MIN(0.5*(B22+B23),$B$4),IF(C23&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C23&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C23,Compose!$A$13:$A$64,1))+(C23-INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C23,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C23,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F22&lt;=0.01,MIN(0.5*(B22+B23),$B$4),IF(C23&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C23&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C23,Compose!$A$15:$A$66,1))+(C23-INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C23,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C23,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E23" s="15">
@@ -6368,11 +6380,11 @@
         <v/>
       </c>
       <c r="G23" s="16">
-        <f>IF(C23&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C23&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C23,Compose!$A$13:$A$64,1))+(C23-INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C23,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C23,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C23&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C23&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C23,Compose!$A$15:$A$66,1))+(C23-INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C23,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C23,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H23" s="16">
-        <f>IF(C23&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C23&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C23,Compose!$A$13:$A$64,1))+(C23-INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C23,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C23,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C23,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C23&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C23&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C23,Compose!$A$15:$A$66,1))+(C23-INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C23,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C23,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C23,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I23" s="20">
@@ -6394,11 +6406,11 @@
         <v/>
       </c>
       <c r="C24" s="16">
-        <f>IF(F23&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F23&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F23,Compose!$G$13:$G$64,1))+(F23-INDEX(Compose!$G$13:$G$64,MATCH(F23,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F23,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F23,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F23,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F23,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F23&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F23&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F23,Compose!$G$15:$G$66,1))+(F23-INDEX(Compose!$G$15:$G$66,MATCH(F23,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F23,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F23,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F23,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F23,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D24" s="16">
-        <f>IF(F23&lt;=0.01,MIN(0.5*(B23+B24),$B$4),IF(C24&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C24&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C24,Compose!$A$13:$A$64,1))+(C24-INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C24,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C24,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F23&lt;=0.01,MIN(0.5*(B23+B24),$B$4),IF(C24&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C24&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C24,Compose!$A$15:$A$66,1))+(C24-INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C24,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C24,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E24" s="15">
@@ -6410,11 +6422,11 @@
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>IF(C24&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C24&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C24,Compose!$A$13:$A$64,1))+(C24-INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C24,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C24,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C24&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C24&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C24,Compose!$A$15:$A$66,1))+(C24-INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C24,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C24,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H24" s="16">
-        <f>IF(C24&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C24&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C24,Compose!$A$13:$A$64,1))+(C24-INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C24,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C24,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C24,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C24&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C24&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C24,Compose!$A$15:$A$66,1))+(C24-INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C24,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C24,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C24,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I24" s="20">
@@ -6436,11 +6448,11 @@
         <v/>
       </c>
       <c r="C25" s="16">
-        <f>IF(F24&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F24&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F24,Compose!$G$13:$G$64,1))+(F24-INDEX(Compose!$G$13:$G$64,MATCH(F24,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F24,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F24,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F24,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F24,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F24&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F24&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F24,Compose!$G$15:$G$66,1))+(F24-INDEX(Compose!$G$15:$G$66,MATCH(F24,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F24,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F24,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F24,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F24,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D25" s="16">
-        <f>IF(F24&lt;=0.01,MIN(0.5*(B24+B25),$B$4),IF(C25&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C25&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C25,Compose!$A$13:$A$64,1))+(C25-INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C25,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C25,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F24&lt;=0.01,MIN(0.5*(B24+B25),$B$4),IF(C25&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C25&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C25,Compose!$A$15:$A$66,1))+(C25-INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C25,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C25,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E25" s="15">
@@ -6452,11 +6464,11 @@
         <v/>
       </c>
       <c r="G25" s="16">
-        <f>IF(C25&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C25&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C25,Compose!$A$13:$A$64,1))+(C25-INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C25,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C25,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C25&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C25&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C25,Compose!$A$15:$A$66,1))+(C25-INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C25,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C25,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H25" s="16">
-        <f>IF(C25&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C25&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C25,Compose!$A$13:$A$64,1))+(C25-INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C25,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C25,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C25,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C25&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C25&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C25,Compose!$A$15:$A$66,1))+(C25-INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C25,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C25,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C25,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I25" s="20">
@@ -6478,11 +6490,11 @@
         <v/>
       </c>
       <c r="C26" s="16">
-        <f>IF(F25&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F25&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F25,Compose!$G$13:$G$64,1))+(F25-INDEX(Compose!$G$13:$G$64,MATCH(F25,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F25,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F25,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F25,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F25,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F25&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F25&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F25,Compose!$G$15:$G$66,1))+(F25-INDEX(Compose!$G$15:$G$66,MATCH(F25,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F25,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F25,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F25,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F25,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D26" s="16">
-        <f>IF(F25&lt;=0.01,MIN(0.5*(B25+B26),$B$4),IF(C26&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C26&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C26,Compose!$A$13:$A$64,1))+(C26-INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C26,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C26,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F25&lt;=0.01,MIN(0.5*(B25+B26),$B$4),IF(C26&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C26&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C26,Compose!$A$15:$A$66,1))+(C26-INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C26,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C26,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E26" s="15">
@@ -6494,11 +6506,11 @@
         <v/>
       </c>
       <c r="G26" s="16">
-        <f>IF(C26&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C26&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C26,Compose!$A$13:$A$64,1))+(C26-INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C26,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C26,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C26&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C26&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C26,Compose!$A$15:$A$66,1))+(C26-INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C26,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C26,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H26" s="16">
-        <f>IF(C26&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C26&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C26,Compose!$A$13:$A$64,1))+(C26-INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C26,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C26,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C26,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C26&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C26&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C26,Compose!$A$15:$A$66,1))+(C26-INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C26,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C26,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C26,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I26" s="20">
@@ -6520,11 +6532,11 @@
         <v/>
       </c>
       <c r="C27" s="16">
-        <f>IF(F26&lt;=INDEX(Compose!$G$13:$G$64,1),INDEX(Compose!$A$13:$A$64,1),IF(F26&gt;=INDEX(Compose!$G$13:$G$64,ROWS(Compose!$G$13:$G$64)),INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$A$13:$A$64,MATCH(F26,Compose!$G$13:$G$64,1))+(F26-INDEX(Compose!$G$13:$G$64,MATCH(F26,Compose!$G$13:$G$64,1)))/(INDEX(Compose!$G$13:$G$64,MATCH(F26,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$G$13:$G$64,MATCH(F26,Compose!$G$13:$G$64,1)))*(INDEX(Compose!$A$13:$A$64,MATCH(F26,Compose!$G$13:$G$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(F26,Compose!$G$13:$G$64,1)))))</f>
+        <f>IF(F26&lt;=INDEX(Compose!$G$15:$G$66,1),INDEX(Compose!$A$15:$A$66,1),IF(F26&gt;=INDEX(Compose!$G$15:$G$66,ROWS(Compose!$G$15:$G$66)),INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$A$15:$A$66,MATCH(F26,Compose!$G$15:$G$66,1))+(F26-INDEX(Compose!$G$15:$G$66,MATCH(F26,Compose!$G$15:$G$66,1)))/(INDEX(Compose!$G$15:$G$66,MATCH(F26,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$G$15:$G$66,MATCH(F26,Compose!$G$15:$G$66,1)))*(INDEX(Compose!$A$15:$A$66,MATCH(F26,Compose!$G$15:$G$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(F26,Compose!$G$15:$G$66,1)))))</f>
         <v/>
       </c>
       <c r="D27" s="16">
-        <f>IF(F26&lt;=0.01,MIN(0.5*(B26+B27),$B$4),IF(C27&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$J$13:$J$64,1),IF(C27&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$J$13:$J$64,ROWS(Compose!$J$13:$J$64)),INDEX(Compose!$J$13:$J$64,MATCH(C27,Compose!$A$13:$A$64,1))+(C27-INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$J$13:$J$64,MATCH(C27,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$J$13:$J$64,MATCH(C27,Compose!$A$13:$A$64,1))))))</f>
+        <f>IF(F26&lt;=0.01,MIN(0.5*(B26+B27),$B$4),IF(C27&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$J$15:$J$66,1),IF(C27&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$J$15:$J$66,ROWS(Compose!$J$15:$J$66)),INDEX(Compose!$J$15:$J$66,MATCH(C27,Compose!$A$15:$A$66,1))+(C27-INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$J$15:$J$66,MATCH(C27,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$J$15:$J$66,MATCH(C27,Compose!$A$15:$A$66,1))))))</f>
         <v/>
       </c>
       <c r="E27" s="15">
@@ -6536,11 +6548,11 @@
         <v/>
       </c>
       <c r="G27" s="16">
-        <f>IF(C27&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$H$13:$H$64,1),IF(C27&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$H$13:$H$64,ROWS(Compose!$H$13:$H$64)),INDEX(Compose!$H$13:$H$64,MATCH(C27,Compose!$A$13:$A$64,1))+(C27-INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$H$13:$H$64,MATCH(C27,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$H$13:$H$64,MATCH(C27,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C27&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$H$15:$H$66,1),IF(C27&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$H$15:$H$66,ROWS(Compose!$H$15:$H$66)),INDEX(Compose!$H$15:$H$66,MATCH(C27,Compose!$A$15:$A$66,1))+(C27-INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$H$15:$H$66,MATCH(C27,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$H$15:$H$66,MATCH(C27,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="H27" s="16">
-        <f>IF(C27&lt;=INDEX(Compose!$A$13:$A$64,1),INDEX(Compose!$I$13:$I$64,1),IF(C27&gt;=INDEX(Compose!$A$13:$A$64,ROWS(Compose!$A$13:$A$64)),INDEX(Compose!$I$13:$I$64,ROWS(Compose!$I$13:$I$64)),INDEX(Compose!$I$13:$I$64,MATCH(C27,Compose!$A$13:$A$64,1))+(C27-INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)))/(INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$A$13:$A$64,MATCH(C27,Compose!$A$13:$A$64,1)))*(INDEX(Compose!$I$13:$I$64,MATCH(C27,Compose!$A$13:$A$64,1)+1)-INDEX(Compose!$I$13:$I$64,MATCH(C27,Compose!$A$13:$A$64,1)))))</f>
+        <f>IF(C27&lt;=INDEX(Compose!$A$15:$A$66,1),INDEX(Compose!$I$15:$I$66,1),IF(C27&gt;=INDEX(Compose!$A$15:$A$66,ROWS(Compose!$A$15:$A$66)),INDEX(Compose!$I$15:$I$66,ROWS(Compose!$I$15:$I$66)),INDEX(Compose!$I$15:$I$66,MATCH(C27,Compose!$A$15:$A$66,1))+(C27-INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)))/(INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$A$15:$A$66,MATCH(C27,Compose!$A$15:$A$66,1)))*(INDEX(Compose!$I$15:$I$66,MATCH(C27,Compose!$A$15:$A$66,1)+1)-INDEX(Compose!$I$15:$I$66,MATCH(C27,Compose!$A$15:$A$66,1)))))</f>
         <v/>
       </c>
       <c r="I27" s="20">

</xml_diff>